<commit_message>
Reviewed documents and crafted individual country sections
</commit_message>
<xml_diff>
--- a/data/assessment/AFE_assessment_2025.xlsx
+++ b/data/assessment/AFE_assessment_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11489" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11441" uniqueCount="222">
   <si>
     <t xml:space="preserve">AFE</t>
   </si>
@@ -686,6 +686,9 @@
     <t xml:space="preserve">Zimbabwe</t>
   </si>
   <si>
+    <t xml:space="preserve">- all -</t>
+  </si>
+  <si>
     <t xml:space="preserve">(empty)</t>
   </si>
   <si>
@@ -758,7 +761,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="17">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -798,20 +801,6 @@
       <left style="medium"/>
       <right style="thin"/>
       <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="thin"/>
-      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
@@ -826,6 +815,27 @@
       <left style="thin"/>
       <right style="medium"/>
       <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="medium"/>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -852,34 +862,6 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium"/>
-      <right style="thin"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
       <right/>
       <top style="thin"/>
       <bottom style="medium"/>
@@ -943,7 +925,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -996,63 +978,47 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="14" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="15" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" xfId="24" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="18" xfId="24" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="19" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -22092,39 +22058,10 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="DataPilot1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" showDrill="0" useAutoFormatting="0" itemPrintTitles="1" indent="0" outline="0" outlineData="0" compact="0" compactData="0">
-  <location ref="A3:D54" firstHeaderRow="1" firstDataRow="1" firstDataCol="3" rowPageCount="1" colPageCount="1"/>
+  <location ref="A3:C40" firstHeaderRow="1" firstDataRow="1" firstDataCol="2" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="20">
     <pivotField compact="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="26">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="22"/>
-      </items>
-    </pivotField>
+    <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
@@ -22184,7 +22121,7 @@
     </pivotField>
     <pivotField axis="axisPage" compact="0" outline="0" showAll="0" defaultSubtotal="0">
       <items count="2">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
       </items>
     </pivotField>
@@ -22194,52 +22131,65 @@
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
   </pivotFields>
-  <rowFields count="3">
-    <field x="1"/>
+  <rowFields count="2">
     <field x="12"/>
     <field x="13"/>
   </rowFields>
-  <rowItems count="51">
+  <rowItems count="37">
     <i>
-      <x v="1"/>
       <x/>
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="2"/>
       <x/>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="4"/>
-      <x v="1"/>
-      <x v="6"/>
     </i>
     <i r="1">
-      <x v="7"/>
+      <x v="1"/>
     </i>
-    <i>
-      <x v="7"/>
-      <x/>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i r="1">
       <x v="14"/>
+    </i>
+    <i r="1">
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="21"/>
     </i>
     <i r="1">
       <x v="22"/>
     </i>
     <i r="1">
-      <x v="1"/>
-      <x v="6"/>
+      <x v="23"/>
     </i>
     <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-      <x/>
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="22"/>
+      <x v="24"/>
     </i>
     <i r="1">
       <x v="25"/>
@@ -22251,7 +22201,22 @@
       <x v="28"/>
     </i>
     <i r="1">
+      <x v="30"/>
+    </i>
+    <i r="1">
+      <x v="32"/>
+    </i>
+    <i r="1">
+      <x v="34"/>
+    </i>
+    <i r="1">
+      <x v="35"/>
+    </i>
+    <i>
       <x v="1"/>
+      <x v="5"/>
+    </i>
+    <i r="1">
       <x v="6"/>
     </i>
     <i r="1">
@@ -22263,128 +22228,24 @@
     <i r="1">
       <x v="26"/>
     </i>
+    <i>
+      <x v="2"/>
+      <x v="3"/>
+    </i>
     <i r="1">
-      <x v="2"/>
       <x v="11"/>
     </i>
-    <i>
-      <x v="10"/>
-      <x v="1"/>
-      <x v="6"/>
+    <i r="1">
+      <x v="20"/>
     </i>
     <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="12"/>
-      <x/>
-      <x v="25"/>
+      <x v="29"/>
     </i>
     <i r="1">
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="13"/>
-      <x/>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="14"/>
-      <x/>
-      <x/>
+      <x v="31"/>
     </i>
     <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="15"/>
-      <x/>
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="22"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="19"/>
-      <x/>
-      <x v="22"/>
-    </i>
-    <i r="1">
-      <x v="25"/>
-    </i>
-    <i r="1">
-      <x v="27"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="35"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="22"/>
-      <x/>
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="23"/>
-      <x/>
-      <x v="22"/>
-    </i>
-    <i r="1">
-      <x v="24"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="25"/>
-      <x/>
-      <x v="27"/>
+      <x v="33"/>
     </i>
     <i t="grand">
       <x/>
@@ -58741,8 +58602,8 @@
   <dimension ref="A1:D54"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="29.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="49.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="37.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.97"/>
   </cols>
@@ -58752,7 +58613,7 @@
         <v>14</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>20</v>
+        <v>219</v>
       </c>
       <c r="C1" s="0"/>
       <c r="D1" s="0"/>
@@ -58765,497 +58626,401 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>219</v>
-      </c>
+      <c r="C3" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="D3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15"/>
+      <c r="B5" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="0"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15"/>
+      <c r="B6" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="0"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15"/>
+      <c r="B7" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="17"/>
+      <c r="D7" s="0"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15"/>
+      <c r="B8" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="17"/>
+      <c r="D8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15"/>
+      <c r="B9" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="0"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15"/>
+      <c r="B10" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="17"/>
+      <c r="D10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15"/>
+      <c r="B11" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="17"/>
+      <c r="D11" s="0"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15"/>
+      <c r="B12" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="0"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15"/>
+      <c r="B13" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="0"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15"/>
+      <c r="B15" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15"/>
+      <c r="B16" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="17"/>
+      <c r="D16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15"/>
+      <c r="B17" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="17"/>
+      <c r="D17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15"/>
+      <c r="B18" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="0"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15"/>
+      <c r="B19" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15"/>
+      <c r="B20" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="17"/>
+      <c r="D20" s="0"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15"/>
+      <c r="B21" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="17"/>
+      <c r="D21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15"/>
+      <c r="B22" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="17"/>
+      <c r="D22" s="0"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15"/>
+      <c r="B23" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="17"/>
+      <c r="D23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15"/>
+      <c r="B24" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="14"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="14"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="16" t="s">
+      <c r="C24" s="17"/>
+      <c r="D24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15"/>
+      <c r="B25" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="0"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15"/>
+      <c r="B26" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="17"/>
+      <c r="D26" s="0"/>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15"/>
+      <c r="B27" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="0"/>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18"/>
+      <c r="B28" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="20"/>
+      <c r="D28" s="0"/>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="B29" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="14"/>
+      <c r="D29" s="0"/>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15"/>
+      <c r="B30" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="17"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19" t="s">
+      <c r="C30" s="17"/>
+      <c r="D30" s="0"/>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15"/>
+      <c r="B31" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="20"/>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="17"/>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="20"/>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21"/>
-      <c r="B10" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="17"/>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="20"/>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="17"/>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="23"/>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="23"/>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="23"/>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="20"/>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21"/>
-      <c r="B17" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="17"/>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="23"/>
-    </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22" t="s">
+      <c r="C31" s="17"/>
+      <c r="D31" s="0"/>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15"/>
+      <c r="B32" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="23"/>
-    </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19" t="s">
+      <c r="C32" s="17"/>
+      <c r="D32" s="0"/>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18"/>
+      <c r="B33" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="20"/>
-    </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18"/>
-      <c r="B21" s="13" t="s">
+      <c r="C33" s="20"/>
+      <c r="D33" s="0"/>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="B34" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="14"/>
+      <c r="D34" s="0"/>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15"/>
+      <c r="B35" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="14"/>
-    </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="17"/>
-    </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="20"/>
-    </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="17"/>
-    </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="20"/>
-    </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" s="14"/>
-    </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="B27" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="D27" s="17"/>
-    </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21"/>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D28" s="23"/>
-    </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="D29" s="20"/>
-    </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="B30" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D30" s="17"/>
-    </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21"/>
-      <c r="B31" s="22"/>
-      <c r="C31" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" s="23"/>
-    </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="20"/>
-    </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21"/>
-      <c r="B33" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D33" s="17"/>
-    </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18"/>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D34" s="20"/>
-    </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="B35" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="0"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21"/>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="D36" s="23"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="17"/>
+      <c r="D36" s="0"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21"/>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="D37" s="23"/>
+      <c r="A37" s="15"/>
+      <c r="B37" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="17"/>
+      <c r="D37" s="0"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21"/>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="D38" s="23"/>
+      <c r="A38" s="15"/>
+      <c r="B38" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C38" s="17"/>
+      <c r="D38" s="0"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21"/>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="D39" s="20"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C39" s="20"/>
+      <c r="D39" s="0"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="21"/>
-      <c r="B40" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D40" s="17"/>
+      <c r="A40" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="B40" s="22"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="0"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18"/>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D41" s="20"/>
+      <c r="A41" s="0"/>
+      <c r="B41" s="0"/>
+      <c r="C41" s="0"/>
+      <c r="D41" s="0"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="B42" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="D42" s="17"/>
+      <c r="A42" s="0"/>
+      <c r="B42" s="0"/>
+      <c r="C42" s="0"/>
+      <c r="D42" s="0"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="21"/>
-      <c r="B43" s="19"/>
-      <c r="C43" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D43" s="20"/>
+      <c r="A43" s="0"/>
+      <c r="B43" s="0"/>
+      <c r="C43" s="0"/>
+      <c r="D43" s="0"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="21"/>
-      <c r="B44" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D44" s="17"/>
+      <c r="A44" s="0"/>
+      <c r="B44" s="0"/>
+      <c r="C44" s="0"/>
+      <c r="D44" s="0"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="21"/>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="D45" s="23"/>
+      <c r="A45" s="0"/>
+      <c r="B45" s="0"/>
+      <c r="C45" s="0"/>
+      <c r="D45" s="0"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="21"/>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="D46" s="23"/>
+      <c r="A46" s="0"/>
+      <c r="B46" s="0"/>
+      <c r="C46" s="0"/>
+      <c r="D46" s="0"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18"/>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D47" s="20"/>
+      <c r="A47" s="0"/>
+      <c r="B47" s="0"/>
+      <c r="C47" s="0"/>
+      <c r="D47" s="0"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
-        <v>202</v>
-      </c>
-      <c r="B48" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="17"/>
+      <c r="A48" s="0"/>
+      <c r="B48" s="0"/>
+      <c r="C48" s="0"/>
+      <c r="D48" s="0"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="21"/>
-      <c r="B49" s="22"/>
-      <c r="C49" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="D49" s="23"/>
+      <c r="A49" s="0"/>
+      <c r="B49" s="0"/>
+      <c r="C49" s="0"/>
+      <c r="D49" s="0"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="21"/>
-      <c r="B50" s="19"/>
-      <c r="C50" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D50" s="20"/>
+      <c r="A50" s="0"/>
+      <c r="B50" s="0"/>
+      <c r="C50" s="0"/>
+      <c r="D50" s="0"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="21"/>
-      <c r="B51" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="D51" s="14"/>
+      <c r="A51" s="0"/>
+      <c r="B51" s="0"/>
+      <c r="C51" s="0"/>
+      <c r="D51" s="0"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="18"/>
-      <c r="B52" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C52" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D52" s="14"/>
+      <c r="A52" s="0"/>
+      <c r="B52" s="0"/>
+      <c r="C52" s="0"/>
+      <c r="D52" s="0"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="B53" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D53" s="14"/>
+      <c r="A53" s="0"/>
+      <c r="B53" s="0"/>
+      <c r="C53" s="0"/>
+      <c r="D53" s="0"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="24" t="s">
-        <v>220</v>
-      </c>
-      <c r="B54" s="25"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="27"/>
+      <c r="A54" s="0"/>
+      <c r="B54" s="0"/>
+      <c r="C54" s="0"/>
+      <c r="D54" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>